<commit_message>
Daily slate 2026-05-07 [auto]
</commit_message>
<xml_diff>
--- a/ui_runner/templates/graded_analysis_tabs_2026-05-05.xlsx
+++ b/ui_runner/templates/graded_analysis_tabs_2026-05-05.xlsx
@@ -471,16 +471,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="E2" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F2" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="n">
-        <v>68.09999999999999</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="3">
@@ -587,16 +587,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="E6" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F6" t="n">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="G6" t="n">
-        <v>42.4</v>
+        <v>39.5</v>
       </c>
     </row>
     <row r="7">
@@ -616,16 +616,16 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="E7" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="F7" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G7" t="n">
-        <v>68.2</v>
+        <v>66.7</v>
       </c>
     </row>
     <row r="8">
@@ -645,16 +645,16 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="E8" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F8" t="n">
         <v>176</v>
       </c>
       <c r="G8" t="n">
-        <v>51.5</v>
+        <v>51.9</v>
       </c>
     </row>
     <row r="9">
@@ -674,16 +674,16 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="E9" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F9" t="n">
         <v>38</v>
       </c>
       <c r="G9" t="n">
-        <v>36.7</v>
+        <v>38.7</v>
       </c>
     </row>
     <row r="10">
@@ -703,16 +703,16 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>689</v>
+        <v>726</v>
       </c>
       <c r="E10" t="n">
-        <v>474</v>
+        <v>496</v>
       </c>
       <c r="F10" t="n">
-        <v>215</v>
+        <v>230</v>
       </c>
       <c r="G10" t="n">
-        <v>68.8</v>
+        <v>68.3</v>
       </c>
     </row>
     <row r="11">
@@ -732,16 +732,16 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="E11" t="n">
         <v>192</v>
       </c>
       <c r="F11" t="n">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="G11" t="n">
-        <v>72.5</v>
+        <v>71.40000000000001</v>
       </c>
     </row>
     <row r="12">
@@ -761,16 +761,16 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="E12" t="n">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F12" t="n">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G12" t="n">
-        <v>69.90000000000001</v>
+        <v>69.8</v>
       </c>
     </row>
     <row r="13">
@@ -790,16 +790,16 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="E13" t="n">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="F13" t="n">
         <v>63</v>
       </c>
       <c r="G13" t="n">
-        <v>64.2</v>
+        <v>64.59999999999999</v>
       </c>
     </row>
     <row r="14">
@@ -819,16 +819,16 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="E14" t="n">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="F14" t="n">
-        <v>113</v>
+        <v>123</v>
       </c>
       <c r="G14" t="n">
-        <v>31.9</v>
+        <v>30.5</v>
       </c>
     </row>
     <row r="15">
@@ -848,16 +848,16 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="E15" t="n">
         <v>20</v>
       </c>
       <c r="F15" t="n">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="G15" t="n">
-        <v>17.1</v>
+        <v>15.9</v>
       </c>
     </row>
     <row r="16">
@@ -906,16 +906,16 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2141</v>
+        <v>2287</v>
       </c>
       <c r="E17" t="n">
-        <v>522</v>
+        <v>545</v>
       </c>
       <c r="F17" t="n">
-        <v>1619</v>
+        <v>1742</v>
       </c>
       <c r="G17" t="n">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
     </row>
   </sheetData>
@@ -1249,7 +1249,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>86</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="C4" t="n">
         <v>86</v>
@@ -1261,13 +1261,13 @@
         <v>92</v>
       </c>
       <c r="F4" t="n">
-        <v>72.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="G4" t="n">
         <v>77</v>
       </c>
       <c r="H4" t="n">
-        <v>63.4</v>
+        <v>64.5</v>
       </c>
       <c r="I4" t="n">
         <v>93</v>
@@ -1291,7 +1291,7 @@
         <v>2</v>
       </c>
       <c r="P4" t="n">
-        <v>34.3</v>
+        <v>35.7</v>
       </c>
       <c r="Q4" t="n">
         <v>70</v>
@@ -1315,10 +1315,10 @@
         <v>1</v>
       </c>
       <c r="X4" t="n">
-        <v>48.9</v>
+        <v>49.4</v>
       </c>
       <c r="Y4" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="AA4" t="n">
         <v>0</v>
@@ -1453,40 +1453,40 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>68.8</v>
+        <v>68.3</v>
       </c>
       <c r="C7" t="n">
-        <v>689</v>
+        <v>726</v>
       </c>
       <c r="D7" t="n">
-        <v>72.5</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="E7" t="n">
-        <v>265</v>
+        <v>269</v>
       </c>
       <c r="F7" t="n">
-        <v>69.90000000000001</v>
+        <v>69.8</v>
       </c>
       <c r="G7" t="n">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="H7" t="n">
-        <v>64.2</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="I7" t="n">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="J7" t="n">
-        <v>31.9</v>
+        <v>30.5</v>
       </c>
       <c r="K7" t="n">
-        <v>166</v>
+        <v>177</v>
       </c>
       <c r="L7" t="n">
-        <v>17.1</v>
+        <v>15.9</v>
       </c>
       <c r="M7" t="n">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="N7" t="n">
         <v>20.8</v>
@@ -1495,16 +1495,16 @@
         <v>24</v>
       </c>
       <c r="P7" t="n">
-        <v>24.4</v>
+        <v>23.8</v>
       </c>
       <c r="Q7" t="n">
-        <v>2141</v>
+        <v>2287</v>
       </c>
       <c r="R7" t="n">
-        <v>68.09999999999999</v>
+        <v>67.3</v>
       </c>
       <c r="S7" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="T7" t="n">
         <v>30</v>
@@ -1513,16 +1513,16 @@
         <v>10</v>
       </c>
       <c r="V7" t="n">
-        <v>42.4</v>
+        <v>39.5</v>
       </c>
       <c r="W7" t="n">
-        <v>33</v>
+        <v>38</v>
       </c>
       <c r="X7" t="n">
-        <v>51.5</v>
+        <v>51.9</v>
       </c>
       <c r="Y7" t="n">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="Z7" t="n">
         <v>100</v>
@@ -1537,16 +1537,16 @@
         <v>14</v>
       </c>
       <c r="AD7" t="n">
-        <v>68.2</v>
+        <v>66.7</v>
       </c>
       <c r="AE7" t="n">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="AF7" t="n">
-        <v>36.7</v>
+        <v>38.7</v>
       </c>
       <c r="AG7" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
     </row>
   </sheetData>

</xml_diff>